<commit_message>
feat(tms): remove express service and special goods pricing rules, update related components
</commit_message>
<xml_diff>
--- a/tms-order/src/main/resources/excel/order_template.xlsx
+++ b/tms-order/src/main/resources/excel/order_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ADMIN\Desktop\DATN\Serp\tms-order\src\main\resources\excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F70A5749-FC17-4743-A32E-1F146CA4626E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9B157133-3375-4B25-A591-20AF0C5B1143}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{DCEF8B10-CC32-4706-81E7-C863D6A361A9}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{DCEF8B10-CC32-4706-81E7-C863D6A361A9}"/>
   </bookViews>
   <sheets>
     <sheet name="Order" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3435" uniqueCount="3414">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3434" uniqueCount="3414">
   <si>
     <t>Phường/xã</t>
   </si>
@@ -11085,7 +11085,7 @@
         <v>3361</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>38</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>6</v>
@@ -11109,9 +11109,6 @@
       </c>
       <c r="B3" s="1" t="s">
         <v>3362</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>38</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>37</v>

</xml_diff>